<commit_message>
update file test case
</commit_message>
<xml_diff>
--- a/manual_test/DuyenNTK Flashcard System Test Case.xlsx
+++ b/manual_test/DuyenNTK Flashcard System Test Case.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Learning24\web\learn-writing-english\manual_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFAED75F-08C4-464A-804E-43AAE1924F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18485ADD-DCB8-4579-AE41-EDE8AD152568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="7" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,12 @@
     <sheet name="Remove all cards" sheetId="6" r:id="rId5"/>
     <sheet name="Shuffle cards" sheetId="7" r:id="rId6"/>
     <sheet name="Download file" sheetId="9" r:id="rId7"/>
-    <sheet name="State Transition" sheetId="2" r:id="rId8"/>
+    <sheet name="Create Note" sheetId="10" r:id="rId8"/>
+    <sheet name="State Transition" sheetId="2" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Create Card'!$A$1:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Create Card'!$A$1:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Create Note'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Delete Card'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Download file'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log In'!$A$1:$H$5</definedName>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="132">
   <si>
     <t>N/A</t>
   </si>
@@ -310,9 +312,6 @@
   <si>
     <t>1.Actor: all users
 2.Users have valid account in the system</t>
-  </si>
-  <si>
-    <t>Vào màn hình đăng nhập thành công</t>
   </si>
   <si>
     <t>Truy cập màn hình đăng nhập</t>
@@ -326,9 +325,6 @@
   </si>
   <si>
     <t>[FlashCard][Log In][UI]Kiểm tra màn hình đúng với thiết kế</t>
-  </si>
-  <si>
-    <t>The account had already been successfully registered.</t>
   </si>
   <si>
     <t>[FlashCard][Log In][Function]Log in account unsuccessfully, in case:
@@ -529,6 +525,84 @@
     <t>The system download file successfully
  - Receive vocabulary.xlsx file includes column such as STT, Từ, IPA, Nghĩa của từ</t>
   </si>
+  <si>
+    <t>1.Actor: all users
+2.Users had already been successfully registered.</t>
+  </si>
+  <si>
+    <t>1.At "Form card" screen, click "Ghi chú" in the dropdown menu
+2.The user chooses &lt;GHI CHÚ&gt; tab
+3.[note] field fill text 
+4.Click on &lt;LƯU&gt; button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Note screen is displayed
+2.Create note screen is displayed
+3.Data is inputted
+4.Created data in the system database.The system shows message:"Thêm dữ liệu thành công!"
+</t>
+  </si>
+  <si>
+    <t>The system shows message:"Thêm dữ liệu thành công!"</t>
+  </si>
+  <si>
+    <t>[FlashCard][Create Note][Function]Create a successful note, in case:
+- Click on &lt;LƯU&gt; button + success</t>
+  </si>
+  <si>
+    <t>[FlashCard][Create Card][Function]Create a unsuccessful card, in case:
+- Click on &lt;THOÁT&gt; button</t>
+  </si>
+  <si>
+    <t>1.User logged in account successfully
+2.Fill data in all fields
+3.Click on &lt;THOÁT&gt; button</t>
+  </si>
+  <si>
+    <t>1.The create card screen is displayed
+2.Data is inputted
+3.The system remove all data in each fields</t>
+  </si>
+  <si>
+    <t>1.At "Form card" screen, click "Ghi chú" in the dropdown menu
+2.The user chooses &lt;GHI CHÚ&gt; tab
+3.[note] field fill text 
+4.Click on &lt;THOÁT&gt; button</t>
+  </si>
+  <si>
+    <t>[FlashCard][Create Note][Function]Create a unsuccessful note, in case:
+- Click on &lt;THOÁT&gt; button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Note screen is displayed
+2.Create note screen is displayed
+3.Data is inputted
+4.The system removes data in [note] fields
+</t>
+  </si>
+  <si>
+    <t>The system removes data in [note] field</t>
+  </si>
+  <si>
+    <t>[FlashCard][Create Note][Function]Create a unsuccessful note, in case:
+- Leave [note] blank</t>
+  </si>
+  <si>
+    <t>1.At "Form card" screen, click "Ghi chú" in the dropdown menu
+2.The user chooses &lt;GHI CHÚ&gt; tab
+3.[note] field is blank 
+4.Click on &lt;LƯU&gt; button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Note screen is displayed
+2.Create note screen is displayed
+3.Data is empty
+4.The system shows message: "Không được để trống!!!"
+</t>
+  </si>
+  <si>
+    <t>The system shows message: "Không được để trống!!!"</t>
+  </si>
 </sst>
 </file>
 
@@ -537,7 +611,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -585,13 +659,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="0"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="7">
@@ -710,7 +777,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -737,9 +804,6 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -752,8 +816,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -764,12 +831,25 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal_Sheet1" xfId="1" xr:uid="{ECE5F156-598F-418F-BB53-741F84C62A4A}"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1281,25 +1361,25 @@
       <c r="A1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1308,7 +1388,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>64</v>
@@ -1334,7 +1414,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>64</v>
@@ -1360,7 +1440,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>64</v>
@@ -1386,7 +1466,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>64</v>
@@ -1412,7 +1492,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>64</v>
@@ -1438,7 +1518,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>64</v>
@@ -1464,7 +1544,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>64</v>
@@ -1489,7 +1569,7 @@
   <autoFilter ref="A1:H8" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="H2:H8">
-    <cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="7" priority="7" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1523,28 +1603,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1561,16 +1641,16 @@
     <row r="3" spans="1:8" ht="126">
       <c r="A3" s="4"/>
       <c r="B3" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>66</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>67</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="10" t="s">
@@ -1595,16 +1675,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="10" t="s">
@@ -1617,19 +1697,19 @@
     <row r="6" spans="1:8" ht="246.6" customHeight="1">
       <c r="A6" s="4"/>
       <c r="B6" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>7</v>
@@ -1643,10 +1723,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>26</v>
@@ -1669,10 +1749,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>28</v>
@@ -1695,10 +1775,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>30</v>
@@ -1721,10 +1801,10 @@
         <v>5</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>32</v>
@@ -1747,10 +1827,10 @@
         <v>6</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>34</v>
@@ -1759,7 +1839,7 @@
         <v>35</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>60</v>
@@ -1773,19 +1853,19 @@
         <v>7</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>7</v>
@@ -1807,7 +1887,7 @@
     <mergeCell ref="A4:H4"/>
   </mergeCells>
   <conditionalFormatting sqref="H3 H5:H12">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H3)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1825,7 +1905,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AEF565D-0726-46E6-AD85-AFA5363204FD}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="59.5546875" customWidth="1"/>
@@ -1837,28 +1917,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" ht="18">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1867,19 +1947,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>50</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -1893,41 +1973,35 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>6</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="11"/>
     </row>
     <row r="4" spans="1:8" ht="90">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="E4" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>55</v>
       </c>
       <c r="F4" s="5" t="s">
@@ -1940,21 +2014,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="108">
+    <row r="5" spans="1:8" ht="90">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>53</v>
+        <v>84</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>52</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>22</v>
@@ -1971,19 +2045,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>105</v>
+        <v>22</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>60</v>
@@ -1997,10 +2071,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>56</v>
@@ -2009,7 +2083,7 @@
         <v>56</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>60</v>
@@ -2018,19 +2092,45 @@
         <v>6</v>
       </c>
     </row>
+    <row r="8" spans="1:8" ht="108">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H7" xr:uid="{7AEF565D-0726-46E6-AD85-AFA5363204FD}"/>
+  <autoFilter ref="A1:H8" xr:uid="{7AEF565D-0726-46E6-AD85-AFA5363204FD}"/>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="H2:H7">
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Failed">
+  <conditionalFormatting sqref="H2:H8">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G7" xr:uid="{08616B86-7664-41E4-8706-DDA43FEB7054}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G8" xr:uid="{08616B86-7664-41E4-8706-DDA43FEB7054}">
       <formula1>"High, Medium, Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H7" xr:uid="{F33A30F3-D26F-4F17-BB0E-F22294474474}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H8" xr:uid="{F33A30F3-D26F-4F17-BB0E-F22294474474}">
       <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2053,28 +2153,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" ht="18">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2083,19 +2183,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>57</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2109,10 +2209,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>58</v>
@@ -2121,7 +2221,7 @@
         <v>59</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>60</v>
@@ -2543,7 +2643,7 @@
   </sheetData>
   <autoFilter ref="A1:H3" xr:uid="{9E3FCD5A-30BD-470A-8DE3-2AF64F04447D}"/>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2574,28 +2674,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" ht="18">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="14" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2604,19 +2704,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>111</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2628,7 +2728,7 @@
   </sheetData>
   <autoFilter ref="A1:H2" xr:uid="{0BB5EB3A-F73A-478B-9305-5AFC908CA8FB}"/>
   <conditionalFormatting sqref="H2">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2659,28 +2759,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" ht="18">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2689,19 +2789,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>115</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2713,7 +2813,7 @@
   </sheetData>
   <autoFilter ref="A1:H2" xr:uid="{E16B402C-C8CC-407E-BD02-EB27480FE176}"/>
   <conditionalFormatting sqref="H2">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2744,28 +2844,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" ht="18">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2774,16 +2874,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="10" t="s">
@@ -2794,12 +2894,12 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="D3" s="16"/>
+      <c r="D3" s="15"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H2" xr:uid="{46AF9C07-F93A-4F0B-96D4-6C3D0DB32A35}"/>
   <conditionalFormatting sqref="H2">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2817,6 +2917,384 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3405550-AA53-4F53-ACED-A7DBB0EE0306}">
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="65.109375" customWidth="1"/>
+    <col min="3" max="3" width="34.21875" customWidth="1"/>
+    <col min="4" max="4" width="40.77734375" customWidth="1"/>
+    <col min="5" max="5" width="39.109375" customWidth="1"/>
+    <col min="6" max="6" width="28.77734375" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="1" customFormat="1" ht="18">
+      <c r="A1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="150" customHeight="1">
+      <c r="A2" s="16">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="144">
+      <c r="A3" s="16">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="162">
+      <c r="A4" s="16">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="18">
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+    </row>
+    <row r="6" spans="1:8" ht="18">
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+    </row>
+    <row r="7" spans="1:8" ht="18">
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+    </row>
+    <row r="8" spans="1:8" ht="18">
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+    </row>
+    <row r="9" spans="1:8" ht="18">
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+    </row>
+    <row r="10" spans="1:8" ht="18">
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+    </row>
+    <row r="11" spans="1:8" ht="18">
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+    </row>
+    <row r="12" spans="1:8" ht="18">
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+    </row>
+    <row r="13" spans="1:8" ht="18">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+    </row>
+    <row r="14" spans="1:8" ht="18">
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+    </row>
+    <row r="15" spans="1:8" ht="18">
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+    </row>
+    <row r="16" spans="1:8" ht="18">
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+    </row>
+    <row r="17" spans="1:8" ht="18">
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+    </row>
+    <row r="18" spans="1:8" ht="18">
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+    </row>
+    <row r="19" spans="1:8" ht="18">
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+    </row>
+    <row r="20" spans="1:8" ht="18">
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+    </row>
+    <row r="21" spans="1:8" ht="18">
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+    </row>
+    <row r="22" spans="1:8" ht="18">
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+    </row>
+    <row r="23" spans="1:8" ht="18">
+      <c r="A23" s="17"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+    </row>
+    <row r="24" spans="1:8" ht="18">
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+    </row>
+    <row r="25" spans="1:8" ht="18">
+      <c r="A25" s="17"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+    </row>
+    <row r="26" spans="1:8" ht="18">
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+    </row>
+    <row r="27" spans="1:8" ht="18">
+      <c r="A27" s="17"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+    </row>
+    <row r="28" spans="1:8" ht="18">
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H4" xr:uid="{B3405550-AA53-4F53-ACED-A7DBB0EE0306}"/>
+  <conditionalFormatting sqref="H2:H4">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Failed">
+      <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G4" xr:uid="{E0D6D318-CBC5-41DB-9877-3E2E9FF17A3F}">
+      <formula1>"High, Medium, Low"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H4" xr:uid="{12927212-B5ED-41B3-9AFC-2F6E60F5082A}">
+      <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B634919C-6A73-48ED-B8C4-3D0E4B88C9C0}">
   <dimension ref="F2:L8"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -2834,14 +3312,14 @@
   <sheetData>
     <row r="2" spans="6:12">
       <c r="F2" s="2"/>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="6:12">
       <c r="F3" s="8" t="s">

</xml_diff>

<commit_message>
update id of sheet log in
</commit_message>
<xml_diff>
--- a/manual_test/DuyenNTK Flashcard System Test Case.xlsx
+++ b/manual_test/DuyenNTK Flashcard System Test Case.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Learning24\web\learn-writing-english\manual_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18485ADD-DCB8-4579-AE41-EDE8AD152568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{961A90A9-F7C9-4A70-9633-F8A4B1CA4932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="1" r:id="rId1"/>
@@ -362,10 +362,6 @@
 - Time: 1h</t>
   </si>
   <si>
-    <t>[FlashCard][Log In][Function]Log in by a invalid access_token unsuccessfully
-- Time &gt; 1h</t>
-  </si>
-  <si>
     <t>[FlashCard][Register][Function]Register account successfully, in case:
 - All fields are valid
 - Navigate to log in page</t>
@@ -602,6 +598,10 @@
   </si>
   <si>
     <t>The system shows message: "Không được để trống!!!"</t>
+  </si>
+  <si>
+    <t>[FlashCard][Log In][Function]Log in by a invalid access_token unsuccessfully
+- Expire time: &gt;= 1h</t>
   </si>
 </sst>
 </file>
@@ -1388,7 +1388,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>64</v>
@@ -1414,7 +1414,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>64</v>
@@ -1440,7 +1440,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>64</v>
@@ -1466,7 +1466,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>64</v>
@@ -1492,7 +1492,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>64</v>
@@ -1518,7 +1518,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>64</v>
@@ -1544,7 +1544,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>64</v>
@@ -1644,7 +1644,7 @@
         <v>67</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>65</v>
@@ -1675,10 +1675,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>25</v>
@@ -1695,21 +1695,23 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="246.6" customHeight="1">
-      <c r="A6" s="4"/>
+      <c r="A6" s="4">
+        <v>2</v>
+      </c>
       <c r="B6" s="5" t="s">
         <v>75</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>74</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>99</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>100</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>7</v>
@@ -1720,13 +1722,13 @@
     </row>
     <row r="7" spans="1:8" ht="90">
       <c r="A7" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>68</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>26</v>
@@ -1746,13 +1748,13 @@
     </row>
     <row r="8" spans="1:8" ht="90">
       <c r="A8" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>69</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>28</v>
@@ -1772,13 +1774,13 @@
     </row>
     <row r="9" spans="1:8" ht="90">
       <c r="A9" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>70</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>30</v>
@@ -1798,13 +1800,13 @@
     </row>
     <row r="10" spans="1:8" ht="103.2" customHeight="1">
       <c r="A10" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>71</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>32</v>
@@ -1824,13 +1826,13 @@
     </row>
     <row r="11" spans="1:8" ht="108">
       <c r="A11" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>72</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>34</v>
@@ -1839,7 +1841,7 @@
         <v>35</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>60</v>
@@ -1850,22 +1852,22 @@
     </row>
     <row r="12" spans="1:8" ht="275.39999999999998" customHeight="1">
       <c r="A12" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>76</v>
+        <v>131</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>74</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>7</v>
@@ -1947,19 +1949,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>50</v>
       </c>
       <c r="E2" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>101</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>102</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -1973,16 +1975,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>123</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="10"/>
@@ -1993,10 +1995,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>51</v>
@@ -2019,10 +2021,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>52</v>
@@ -2045,10 +2047,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>53</v>
@@ -2071,10 +2073,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>56</v>
@@ -2083,7 +2085,7 @@
         <v>56</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>60</v>
@@ -2097,10 +2099,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>56</v>
@@ -2109,7 +2111,7 @@
         <v>56</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>60</v>
@@ -2183,19 +2185,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>57</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2209,10 +2211,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>58</v>
@@ -2221,7 +2223,7 @@
         <v>59</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>60</v>
@@ -2704,19 +2706,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>109</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2789,19 +2791,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="5" t="s">
         <v>112</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>113</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2874,16 +2876,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>114</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>115</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="10" t="s">
@@ -2961,19 +2963,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>118</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>119</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2987,19 +2989,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>127</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>60</v>
@@ -3013,19 +3015,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>130</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>131</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
add search word sheet
</commit_message>
<xml_diff>
--- a/manual_test/DuyenNTK Flashcard System Test Case.xlsx
+++ b/manual_test/DuyenNTK Flashcard System Test Case.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Learning24\web\learn-writing-english\manual_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27F0D958-CE7D-4EC0-9858-306B39358460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B30C1F5-0749-4EC2-94BA-A327AF628AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="10" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="1" r:id="rId1"/>
@@ -18,24 +18,27 @@
     <sheet name="Create Card" sheetId="4" r:id="rId3"/>
     <sheet name="Delete Card" sheetId="5" r:id="rId4"/>
     <sheet name="View list card" sheetId="12" r:id="rId5"/>
-    <sheet name="Remove all cards" sheetId="6" r:id="rId6"/>
-    <sheet name="Shuffle cards" sheetId="7" r:id="rId7"/>
-    <sheet name="Download file" sheetId="9" r:id="rId8"/>
-    <sheet name="Create Note" sheetId="10" r:id="rId9"/>
-    <sheet name="Delete Note" sheetId="11" r:id="rId10"/>
-    <sheet name="View list notes" sheetId="13" r:id="rId11"/>
-    <sheet name="State Transition" sheetId="2" r:id="rId12"/>
+    <sheet name="Search card" sheetId="14" r:id="rId6"/>
+    <sheet name="Remove all cards" sheetId="6" r:id="rId7"/>
+    <sheet name="Shuffle cards" sheetId="7" r:id="rId8"/>
+    <sheet name="Download file" sheetId="9" r:id="rId9"/>
+    <sheet name="Create Note" sheetId="10" r:id="rId10"/>
+    <sheet name="Delete Note" sheetId="11" r:id="rId11"/>
+    <sheet name="View list notes" sheetId="13" r:id="rId12"/>
+    <sheet name="State Transition" sheetId="2" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Create Card'!$A$1:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Create Note'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Create Note'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Delete Card'!$A$1:$H$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Delete Note'!$A$1:$H$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Download file'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Delete Note'!$A$1:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Download file'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log In'!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Register!$A$1:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Remove all cards'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Shuffle cards'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Remove all cards'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Search card'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Shuffle cards'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'View list card'!$A$1:$H$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="149">
   <si>
     <t>N/A</t>
   </si>
@@ -670,6 +673,29 @@
   <si>
     <t>1.Form Card screen is displayed
 2.It will rotate 2 sides.</t>
+  </si>
+  <si>
+    <t>Search word successfully</t>
+  </si>
+  <si>
+    <t>1.User logged in account successfully
+2.Fill data in all fields
+ + [new_word] field inputs "search(v)"
+ + [mean_of_word] field inputs "tìm kiếm", 
+ + [ipa_text] field inputs "sɝːtʃ"     
+ + [new_word] field inputs "fix(v)"
+ + [mean_of_word] field inputs "sửa chữa", 
+ + [ipa_text] field inputs "fɪks" 
+3.Click on &lt;LƯU&gt; button
+4.Enter search key: "fix"
+5.Click &lt;close&gt; icon in the search bar</t>
+  </si>
+  <si>
+    <t>1.The create card screen is displayed
+2.Data is inputted
+3.Created data in the system, and show in card list.The system shows message: "Thêm dữ liệu thành công"
+4.Show the first search result with card title "fix"
+5.The system will remove text "fix"</t>
   </si>
 </sst>
 </file>
@@ -907,7 +933,17 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal_Sheet1" xfId="1" xr:uid="{ECE5F156-598F-418F-BB53-741F84C62A4A}"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1667,7 +1703,7 @@
   <autoFilter ref="A1:H8" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="H2:H8">
-    <cfRule type="containsText" dxfId="10" priority="7" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="11" priority="7" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1684,6 +1720,384 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3405550-AA53-4F53-ACED-A7DBB0EE0306}">
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="65.109375" customWidth="1"/>
+    <col min="3" max="3" width="34.21875" customWidth="1"/>
+    <col min="4" max="4" width="40.77734375" customWidth="1"/>
+    <col min="5" max="5" width="39.109375" customWidth="1"/>
+    <col min="6" max="6" width="28.77734375" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="1" customFormat="1" ht="18">
+      <c r="A1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="150" customHeight="1">
+      <c r="A2" s="16">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="144">
+      <c r="A3" s="16">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="162">
+      <c r="A4" s="16">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="18">
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+    </row>
+    <row r="6" spans="1:8" ht="18">
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+    </row>
+    <row r="7" spans="1:8" ht="18">
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+    </row>
+    <row r="8" spans="1:8" ht="18">
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+    </row>
+    <row r="9" spans="1:8" ht="18">
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+    </row>
+    <row r="10" spans="1:8" ht="18">
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+    </row>
+    <row r="11" spans="1:8" ht="18">
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+    </row>
+    <row r="12" spans="1:8" ht="18">
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+    </row>
+    <row r="13" spans="1:8" ht="18">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+    </row>
+    <row r="14" spans="1:8" ht="18">
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+    </row>
+    <row r="15" spans="1:8" ht="18">
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+    </row>
+    <row r="16" spans="1:8" ht="18">
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+    </row>
+    <row r="17" spans="1:8" ht="18">
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+    </row>
+    <row r="18" spans="1:8" ht="18">
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+    </row>
+    <row r="19" spans="1:8" ht="18">
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+    </row>
+    <row r="20" spans="1:8" ht="18">
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+    </row>
+    <row r="21" spans="1:8" ht="18">
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+    </row>
+    <row r="22" spans="1:8" ht="18">
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+    </row>
+    <row r="23" spans="1:8" ht="18">
+      <c r="A23" s="17"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+    </row>
+    <row r="24" spans="1:8" ht="18">
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+    </row>
+    <row r="25" spans="1:8" ht="18">
+      <c r="A25" s="17"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+    </row>
+    <row r="26" spans="1:8" ht="18">
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+    </row>
+    <row r="27" spans="1:8" ht="18">
+      <c r="A27" s="17"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+    </row>
+    <row r="28" spans="1:8" ht="18">
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H4" xr:uid="{B3405550-AA53-4F53-ACED-A7DBB0EE0306}"/>
+  <conditionalFormatting sqref="H2:H4">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Failed">
+      <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G4" xr:uid="{E0D6D318-CBC5-41DB-9877-3E2E9FF17A3F}">
+      <formula1>"High, Medium, Low"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H4" xr:uid="{12927212-B5ED-41B3-9AFC-2F6E60F5082A}">
+      <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAB543C6-00AF-4117-A1A7-12E5C04D656D}">
   <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -2035,7 +2449,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FDF424E-1868-4D09-806D-40F6151E0D4F}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -2117,7 +2531,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B634919C-6A73-48ED-B8C4-3D0E4B88C9C0}">
   <dimension ref="F2:L8"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -2595,7 +3009,7 @@
     <mergeCell ref="A4:H4"/>
   </mergeCells>
   <conditionalFormatting sqref="H3 H5:H12">
-    <cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H3)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2830,7 +3244,7 @@
   <autoFilter ref="A1:H8" xr:uid="{7AEF565D-0726-46E6-AD85-AFA5363204FD}"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="H2:H8">
-    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3351,7 +3765,7 @@
   </sheetData>
   <autoFilter ref="A1:H3" xr:uid="{9E3FCD5A-30BD-470A-8DE3-2AF64F04447D}"/>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3432,8 +3846,9 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H2" xr:uid="{70D05D1E-01D1-4596-9CF6-9E1A7DB14A57}"/>
   <conditionalFormatting sqref="H2">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3450,6 +3865,91 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09F608BF-4A7F-41ED-AECC-DEF15F05F8FC}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="45.21875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="29.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="42.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="32.109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="25.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.88671875" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="342">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F2" s="5"/>
+      <c r="G2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H2" xr:uid="{09F608BF-4A7F-41ED-AECC-DEF15F05F8FC}"/>
+  <conditionalFormatting sqref="H2">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Failed">
+      <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{DC435498-22B7-4243-ABF0-99FEC7556E06}">
+      <formula1>"High, Medium, Low"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{BCBAF0A5-7940-453E-AF73-009A88EFD84C}">
+      <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BB5EB3A-F73A-478B-9305-5AFC908CA8FB}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -3534,7 +4034,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E16B402C-C8CC-407E-BD02-EB27480FE176}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -3619,7 +4119,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF9C07-F93A-4F0B-96D4-6C3D0DB32A35}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -3704,382 +4204,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3405550-AA53-4F53-ACED-A7DBB0EE0306}">
-  <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="2" max="2" width="65.109375" customWidth="1"/>
-    <col min="3" max="3" width="34.21875" customWidth="1"/>
-    <col min="4" max="4" width="40.77734375" customWidth="1"/>
-    <col min="5" max="5" width="39.109375" customWidth="1"/>
-    <col min="6" max="6" width="28.77734375" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" ht="18">
-      <c r="A1" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" s="12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="150" customHeight="1">
-      <c r="A2" s="16">
-        <v>1</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="144">
-      <c r="A3" s="16">
-        <v>2</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="162">
-      <c r="A4" s="16">
-        <v>3</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="18">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-    </row>
-    <row r="6" spans="1:8" ht="18">
-      <c r="A6" s="17"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-    </row>
-    <row r="7" spans="1:8" ht="18">
-      <c r="A7" s="17"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-    </row>
-    <row r="8" spans="1:8" ht="18">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-    </row>
-    <row r="9" spans="1:8" ht="18">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-    </row>
-    <row r="10" spans="1:8" ht="18">
-      <c r="A10" s="17"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-    </row>
-    <row r="11" spans="1:8" ht="18">
-      <c r="A11" s="17"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-    </row>
-    <row r="12" spans="1:8" ht="18">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-    </row>
-    <row r="13" spans="1:8" ht="18">
-      <c r="A13" s="17"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-    </row>
-    <row r="14" spans="1:8" ht="18">
-      <c r="A14" s="17"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-    </row>
-    <row r="15" spans="1:8" ht="18">
-      <c r="A15" s="17"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
-    </row>
-    <row r="16" spans="1:8" ht="18">
-      <c r="A16" s="17"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-    </row>
-    <row r="17" spans="1:8" ht="18">
-      <c r="A17" s="17"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-    </row>
-    <row r="18" spans="1:8" ht="18">
-      <c r="A18" s="17"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-    </row>
-    <row r="19" spans="1:8" ht="18">
-      <c r="A19" s="17"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
-    </row>
-    <row r="20" spans="1:8" ht="18">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-    </row>
-    <row r="21" spans="1:8" ht="18">
-      <c r="A21" s="17"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="17"/>
-    </row>
-    <row r="22" spans="1:8" ht="18">
-      <c r="A22" s="17"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
-    </row>
-    <row r="23" spans="1:8" ht="18">
-      <c r="A23" s="17"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-    </row>
-    <row r="24" spans="1:8" ht="18">
-      <c r="A24" s="17"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
-    </row>
-    <row r="25" spans="1:8" ht="18">
-      <c r="A25" s="17"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-    </row>
-    <row r="26" spans="1:8" ht="18">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-    </row>
-    <row r="27" spans="1:8" ht="18">
-      <c r="A27" s="17"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="17"/>
-    </row>
-    <row r="28" spans="1:8" ht="18">
-      <c r="A28" s="17"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="17"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H4" xr:uid="{B3405550-AA53-4F53-ACED-A7DBB0EE0306}"/>
-  <conditionalFormatting sqref="H2:H4">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Failed">
-      <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G4" xr:uid="{E0D6D318-CBC5-41DB-9877-3E2E9FF17A3F}">
-      <formula1>"High, Medium, Low"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H4" xr:uid="{12927212-B5ED-41B3-9AFC-2F6E60F5082A}">
-      <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
update some test case
</commit_message>
<xml_diff>
--- a/manual_test/DuyenNTK Flashcard System Test Case.xlsx
+++ b/manual_test/DuyenNTK Flashcard System Test Case.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Learning24\web\learn-writing-english\manual_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B30C1F5-0749-4EC2-94BA-A327AF628AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F423D2A-4EF1-49AE-8CC7-82A5E7B01B0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="1" r:id="rId1"/>
@@ -39,6 +39,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Search card'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Shuffle cards'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'View list card'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'View list notes'!$A$1:$H$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -324,13 +325,6 @@
     <t>Truy cập màn hình đăng nhập</t>
   </si>
   <si>
-    <t>Màn hình đăng nhập được hiển thị đúng như trong thiết kế
-trong đó có các thông tin bắt buộc:
- - Textbox [email] là bắt buộc
- - Textbox [password] là bắt buộc và icon ẩn/hiện 
- - Button &lt;Đăng nhập&gt;</t>
-  </si>
-  <si>
     <t>[FlashCard][Log In][UI]Kiểm tra màn hình đúng với thiết kế</t>
   </si>
   <si>
@@ -475,11 +469,6 @@
     <t>1.The system shows json detail of user</t>
   </si>
   <si>
-    <t>1.Create card screen is displayed
-2.Data is inputted
-3.Created data in the system, and show in card list.The system shows message: "Thêm dữ liệu thành công"</t>
-  </si>
-  <si>
     <t>The system shows message: "Thêm dữ liệu thành công"</t>
   </si>
   <si>
@@ -487,10 +476,6 @@
   </si>
   <si>
     <t>The system shows dialog and remove a card in UI &amp; database</t>
-  </si>
-  <si>
-    <t>1.Confirmation dialog "Bạn có chắc là muốn xóa không ?" is displayed
-2.The system will remove a card in UI &amp; database</t>
   </si>
   <si>
     <t>The system shows dialog and don't remove a card in UI &amp; database</t>
@@ -498,10 +483,6 @@
   <si>
     <t>1.The user was created some cards
 2.Click &lt;XÓA TẤT CẢ&gt; button</t>
-  </si>
-  <si>
-    <t>1.The list card shows all cards
-2.The system remove all cards in UI &amp; database.</t>
   </si>
   <si>
     <t>The system remove all cards in UI &amp; database.</t>
@@ -696,6 +677,29 @@
 3.Created data in the system, and show in card list.The system shows message: "Thêm dữ liệu thành công"
 4.Show the first search result with card title "fix"
 5.The system will remove text "fix"</t>
+  </si>
+  <si>
+    <t>1.Create card screen is displayed
+2.Data is inputted
+3.Created data in the system, and show in card list.The system shows message: "Thêm dữ liệu thành công"
+ + The number of cards has increased on the badge</t>
+  </si>
+  <si>
+    <t>1.Confirmation dialog "Bạn có chắc là muốn xóa không ?" is displayed
+2.The system will remove a card in UI &amp; database
+ + The number of cards has decreased on the badge.</t>
+  </si>
+  <si>
+    <t>1.The list card shows all cards
+2.The system remove all cards in UI &amp; database.
+ + The number of cards has decreased on the badge.</t>
+  </si>
+  <si>
+    <t>Màn hình đăng nhập được hiển thị đúng như trong thiết kế
+trong đó có các thông tin bắt buộc:
+ - Textbox [email] is mandatory
+ - Textbox [password] with &lt;eye&gt; icon is mandatory
+ - Button &lt;ĐĂNG NHẬP&gt;</t>
   </si>
 </sst>
 </file>
@@ -1522,7 +1526,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>64</v>
@@ -1548,7 +1552,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>64</v>
@@ -1574,7 +1578,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>64</v>
@@ -1600,7 +1604,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>64</v>
@@ -1626,7 +1630,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>64</v>
@@ -1652,7 +1656,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>64</v>
@@ -1678,7 +1682,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>64</v>
@@ -1764,19 +1768,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -1790,19 +1794,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>60</v>
@@ -1816,19 +1820,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>60</v>
@@ -2080,7 +2084,7 @@
   </sheetData>
   <autoFilter ref="A1:H4" xr:uid="{B3405550-AA53-4F53-ACED-A7DBB0EE0306}"/>
   <conditionalFormatting sqref="H2:H4">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2142,19 +2146,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2168,19 +2172,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>60</v>
@@ -2432,7 +2436,7 @@
   </sheetData>
   <autoFilter ref="A1:H3" xr:uid="{B3405550-AA53-4F53-ACED-A7DBB0EE0306}"/>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2494,16 +2498,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
@@ -2514,8 +2518,9 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H2" xr:uid="{6FDF424E-1868-4D09-806D-40F6151E0D4F}"/>
   <conditionalFormatting sqref="H2">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2761,16 +2766,16 @@
     <row r="3" spans="1:8" ht="126">
       <c r="A3" s="4"/>
       <c r="B3" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>65</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>66</v>
+        <v>148</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="10" t="s">
@@ -2795,16 +2800,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="10" t="s">
@@ -2819,19 +2824,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>98</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>99</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>7</v>
@@ -2845,10 +2850,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>26</v>
@@ -2871,10 +2876,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>28</v>
@@ -2897,10 +2902,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>30</v>
@@ -2923,10 +2928,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>32</v>
@@ -2949,10 +2954,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>34</v>
@@ -2961,7 +2966,7 @@
         <v>35</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>60</v>
@@ -2975,19 +2980,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>7</v>
@@ -3064,24 +3069,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="144">
+    <row r="2" spans="1:8" ht="199.8" customHeight="1">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>50</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -3095,16 +3100,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="10"/>
@@ -3115,10 +3120,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>51</v>
@@ -3141,10 +3146,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>52</v>
@@ -3167,10 +3172,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>53</v>
@@ -3193,10 +3198,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>56</v>
@@ -3205,7 +3210,7 @@
         <v>56</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>60</v>
@@ -3219,10 +3224,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>56</v>
@@ -3231,7 +3236,7 @@
         <v>56</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>60</v>
@@ -3300,24 +3305,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="90">
+    <row r="2" spans="1:8" ht="144">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>57</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>104</v>
+        <v>146</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -3331,10 +3336,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>58</v>
@@ -3343,7 +3348,7 @@
         <v>59</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>60</v>
@@ -3826,16 +3831,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
@@ -3911,16 +3916,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
@@ -3933,7 +3938,7 @@
   </sheetData>
   <autoFilter ref="A1:H2" xr:uid="{09F608BF-4A7F-41ED-AECC-DEF15F05F8FC}"/>
   <conditionalFormatting sqref="H2">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3989,24 +3994,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="72">
+    <row r="2" spans="1:8" ht="108">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>107</v>
+        <v>147</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -4018,7 +4023,7 @@
   </sheetData>
   <autoFilter ref="A1:H2" xr:uid="{0BB5EB3A-F73A-478B-9305-5AFC908CA8FB}"/>
   <conditionalFormatting sqref="H2">
-    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4079,19 +4084,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -4103,7 +4108,7 @@
   </sheetData>
   <autoFilter ref="A1:H2" xr:uid="{E16B402C-C8CC-407E-BD02-EB27480FE176}"/>
   <conditionalFormatting sqref="H2">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4164,16 +4169,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="10" t="s">
@@ -4189,7 +4194,7 @@
   </sheetData>
   <autoFilter ref="A1:H2" xr:uid="{46AF9C07-F93A-4F0B-96D4-6C3D0DB32A35}"/>
   <conditionalFormatting sqref="H2">
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
update file log in test case
</commit_message>
<xml_diff>
--- a/manual_test/DuyenNTK Flashcard System Test Case.xlsx
+++ b/manual_test/DuyenNTK Flashcard System Test Case.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Learning24\web\learn-writing-english\manual_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7AA6261-7ADA-4DE1-A3BF-1384B8BCDADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57269D8-17FA-425E-9E72-A88C9044CB75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="9" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="1" r:id="rId1"/>
@@ -34,8 +34,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Delete Card'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Delete Note'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Download file'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log In'!$A$1:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Register!$A$1:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log In'!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Register!$A$1:$I$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Remove all cards'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Remove all notes'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Search card'!$A$1:$H$2</definedName>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="179">
   <si>
     <t>N/A</t>
   </si>
@@ -158,53 +158,28 @@
 3.Click on &lt;ĐĂNG NHẬP&gt; button</t>
   </si>
   <si>
-    <t>1.Users access the system
-2.All fields are empty
-3.Click on &lt;ĐĂNG NHẬP&gt; button</t>
-  </si>
-  <si>
     <t>1.Log In screen is displayed
 2.Data is empty
 3.User log in unsuccessfully
  - The system shows message: "Không được để trống"</t>
   </si>
   <si>
-    <t>1.Users access the system
-2.[email] field is blank
-3.Click on &lt;ĐĂNG NHẬP&gt; button</t>
-  </si>
-  <si>
     <t>1.Log In screen is displayed
 2.[email] field is blank
 3.User log in unsuccessfully
  - The system shows message: "Không được để trống"</t>
   </si>
   <si>
-    <t>1.Users access the system
-2.[password] field is blank
-3.Click on &lt;ĐĂNG NHẬP&gt; button</t>
-  </si>
-  <si>
     <t>1.Log In screen is displayed
 2.[password] field is blank
 3.User log in unsuccessfully
  - The system shows message: "Không được để trống"</t>
   </si>
   <si>
-    <t>1.Users access the system
-2.[password] field length is less than 8
-3.Click on &lt;ĐĂNG NHẬP&gt; button</t>
-  </si>
-  <si>
     <t>1.Log In screen is displayed
 2.Data is inputted
 3.User log in unsuccessfully
  - The system shows message: "Mật khẩu phải tối thiểu 8 ký tự!"</t>
-  </si>
-  <si>
-    <t>1.Users access the system
-2.[email] field is not existed in database
-3.Click on &lt;ĐĂNG NHẬP&gt; button</t>
   </si>
   <si>
     <t>1.Log In screen is displayed
@@ -359,10 +334,6 @@
   </si>
   <si>
     <t>[FlashCard][Register][Function]Register account unsuccessfully, in case:
-- Leave [username] &amp; [username] &amp; [email] &amp; [password] are blank</t>
-  </si>
-  <si>
-    <t>[FlashCard][Register][Function]Register account unsuccessfully, in case:
 - Leave [username] blank</t>
   </si>
   <si>
@@ -378,11 +349,6 @@
 - Length of password &lt; 8</t>
   </si>
   <si>
-    <t>[FlashCard][Register][Function]Register account unsuccessfully
-- Input [email] is invalid
-(11111111@gmail.com, 1@gmail.com, abc123@example.com)</t>
-  </si>
-  <si>
     <t>1.Actor: all users
 2.Users have logged into system</t>
   </si>
@@ -429,10 +395,6 @@
   <si>
     <t>[FlashCard][Download file][Function]Download file successfully, in case:
 - Click on &lt;TẢI FILE&gt; button</t>
-  </si>
-  <si>
-    <t>[FlashCard][Log In][Function]Log in successfully
- - Click on &lt;ĐĂNG NHẬP&gt; button success</t>
   </si>
   <si>
     <t>The system shows message: "Tài khoản không tồn tại!Bạn chưa đăng ký!!!"</t>
@@ -779,6 +741,111 @@
   </si>
   <si>
     <t>Link "Đi đến trang tìm từ để lấy phiên âm quốc tế chuẩn"</t>
+  </si>
+  <si>
+    <t>Test data</t>
+  </si>
+  <si>
+    <t>[FlashCard][Register][Function]Register account unsuccessfully
+- Input [email] is invalid</t>
+  </si>
+  <si>
+    <t>[FlashCard][Register][Function]Register account unsuccessfully, in case:
+- Leave [username] &amp; [email] &amp; [password] are blank</t>
+  </si>
+  <si>
+    <t>[FlashCard][Log In][Function]Log in account unsuccessfully
+- [email] field is invalid</t>
+  </si>
+  <si>
+    <t>1.Actor: all users
+2.User is not sign up account.</t>
+  </si>
+  <si>
+    <t>1.Log In screen is displayed
+2.Data is inputted
+3.User log in unsuccessfully
+ - The system shows message: "Định dạng email không hợp lệ!"</t>
+  </si>
+  <si>
+    <t>[FlashCard][Log In][Function]Log in account unsuccessfully
+- [email] field is valid
+- [password] field is wrong</t>
+  </si>
+  <si>
+    <t>email: testapp@gmail.com
+password: 6543217890</t>
+  </si>
+  <si>
+    <t>1.Log In screen is displayed
+2.Data is inputted
+3.User log in unsuccessfully
+ - The system shows message: "Email or password không đúng!"</t>
+  </si>
+  <si>
+    <t>The system doesn't have message</t>
+  </si>
+  <si>
+    <t>Local part: 
+ + admin, hello
+Full email:
+ + user.@example.com
+ + user..name@example.com
+ + user@@example.com
+ + user@@example.com
+ + user@.com
+ + user@com
+ + user name@example.com
+ + user@192.168.1.999
+ + user@exam_ple.com</t>
+  </si>
+  <si>
+    <t>[FlashCard][Log In][Function]Log in successfully
+ - Click on &lt;ĐĂNG NHẬP&gt; button + success</t>
+  </si>
+  <si>
+    <t>[FlashCard][Log In][Function]Log in successfully
+ - Press enter &lt;ĐĂNG NHẬP&gt; button + success</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.Click [email] field inputs data --&gt; enter --&gt; [password] field inputs data
+3.Press enter &lt;ĐĂNG NHẬP&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[email] field is blank
+3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.All fields are empty
+3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[password] field is blank
+3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[password] field length is less than 8
+3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[email] field is not existed in database
+3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[email] field is invalid
+3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[email] field is valid, [password] field is wrong
+3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
   </si>
 </sst>
 </file>
@@ -954,7 +1021,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1022,6 +1089,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1582,241 +1652,251 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="57.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="43.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="47" style="1" customWidth="1"/>
-    <col min="5" max="5" width="45.44140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="23.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="17.77734375" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="4" width="43.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="47" style="1" customWidth="1"/>
+    <col min="6" max="6" width="45.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="23.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="17.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="17.77734375" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>158</v>
       </c>
       <c r="E1" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="H1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="I1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="126">
+    <row r="2" spans="1:9" ht="126">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D2" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="5"/>
+      <c r="E2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>145</v>
-      </c>
       <c r="F2" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="H2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="I2" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="90">
+    <row r="3" spans="1:9" ht="90">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>73</v>
+        <v>160</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I3" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="90">
+    <row r="4" spans="1:9" ht="90">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="90">
+    <row r="5" spans="1:9" ht="90">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I5" s="11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="90">
+    <row r="6" spans="1:9" ht="90">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D6" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="108">
+    <row r="7" spans="1:9" ht="108">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D7" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="108">
+    <row r="8" spans="1:9" ht="108">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>78</v>
+        <v>159</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D8" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" s="11" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H8" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}"/>
+  <autoFilter ref="A1:I8" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}"/>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="H2:H8">
+  <conditionalFormatting sqref="I2:I8">
     <cfRule type="containsText" dxfId="12" priority="7" operator="containsText" text="Failed">
-      <formula>NOT(ISERROR(SEARCH("Failed",H2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Failed",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H8" xr:uid="{0FBBFA33-30F5-4E0C-9516-B35814C9A72D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I8" xr:uid="{0FBBFA33-30F5-4E0C-9516-B35814C9A72D}">
       <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G8" xr:uid="{455278D2-97C7-4EB1-A089-10A454F8270A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H8" xr:uid="{455278D2-97C7-4EB1-A089-10A454F8270A}">
       <formula1>"High, Medium, Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1843,13 +1923,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
@@ -1867,22 +1947,22 @@
     <row r="2" spans="1:8" s="1" customFormat="1" ht="283.2" customHeight="1">
       <c r="A2" s="19"/>
       <c r="B2" s="20" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H2" s="11" t="s">
         <v>12</v>
@@ -1893,19 +1973,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>7</v>
@@ -1919,22 +1999,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>6</v>
@@ -1945,22 +2025,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>6</v>
@@ -1971,22 +2051,22 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>6</v>
@@ -2261,13 +2341,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
@@ -2287,19 +2367,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2313,22 +2393,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H3" s="11" t="s">
         <v>6</v>
@@ -2611,13 +2691,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>2</v>
@@ -2637,19 +2717,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2696,13 +2776,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
@@ -2722,16 +2802,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
@@ -2779,7 +2859,7 @@
     <row r="2" spans="6:12">
       <c r="F2" s="2"/>
       <c r="G2" s="25" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H2" s="25"/>
       <c r="I2" s="25"/>
@@ -2789,33 +2869,33 @@
     </row>
     <row r="3" spans="6:12">
       <c r="F3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="4" spans="6:12">
       <c r="F4" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>0</v>
@@ -2835,13 +2915,13 @@
     </row>
     <row r="5" spans="6:12">
       <c r="F5" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>0</v>
@@ -2858,7 +2938,7 @@
     </row>
     <row r="6" spans="6:12">
       <c r="F6" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>0</v>
@@ -2867,13 +2947,13 @@
         <v>0</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>0</v>
@@ -2881,7 +2961,7 @@
     </row>
     <row r="7" spans="6:12">
       <c r="F7" s="3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>0</v>
@@ -2893,7 +2973,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>0</v>
@@ -2904,7 +2984,7 @@
     </row>
     <row r="8" spans="6:12">
       <c r="F8" s="3" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>0</v>
@@ -2922,7 +3002,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -2937,47 +3017,50 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1472075-90BA-4648-91D3-5DF1C222D637}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="48.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="42.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="47.21875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="58.44140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="50.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="53" style="1" customWidth="1"/>
+    <col min="3" max="4" width="42.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="47.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="58.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="50.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5546875" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>158</v>
       </c>
       <c r="E1" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="H1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="I1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1">
+    <row r="2" spans="1:9" hidden="1">
       <c r="A2" s="22"/>
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
@@ -2985,31 +3068,33 @@
       <c r="E2" s="23"/>
       <c r="F2" s="23"/>
       <c r="G2" s="23"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="3" spans="1:8" ht="162">
+      <c r="H2" s="23"/>
+      <c r="I2" s="24"/>
+    </row>
+    <row r="3" spans="1:9" ht="162">
       <c r="A3" s="4"/>
       <c r="B3" s="5" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>151</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="D3" s="5"/>
       <c r="E3" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H3" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I3" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1">
+    <row r="4" spans="1:9" hidden="1">
       <c r="A4" s="22"/>
       <c r="B4" s="23"/>
       <c r="C4" s="23"/>
@@ -3017,216 +3102,312 @@
       <c r="E4" s="23"/>
       <c r="F4" s="23"/>
       <c r="G4" s="23"/>
-      <c r="H4" s="24"/>
-    </row>
-    <row r="5" spans="1:8" ht="94.8" customHeight="1">
+      <c r="H4" s="23"/>
+      <c r="I4" s="24"/>
+    </row>
+    <row r="5" spans="1:9" ht="94.8" customHeight="1">
       <c r="A5" s="4">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>91</v>
+        <v>169</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D5" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="10" t="s">
+      <c r="F5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G5" s="6"/>
+      <c r="H5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="I5" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="246.6" customHeight="1">
+    <row r="6" spans="1:9" ht="109.2" customHeight="1">
       <c r="A6" s="4">
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>71</v>
+        <v>170</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>70</v>
+        <v>100</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>165</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="G6" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="6"/>
+      <c r="H6" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="246.6" customHeight="1">
+      <c r="A7" s="4">
+        <v>2</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="H7" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="I7" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="90">
-      <c r="A7" s="4">
+    <row r="8" spans="1:9" ht="90">
+      <c r="A8" s="4">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="B8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="G8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="90">
+      <c r="A9" s="4">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="F9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H7" s="11" t="s">
+      <c r="H9" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I9" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="90">
-      <c r="A8" s="4">
-        <v>4</v>
-      </c>
-      <c r="B8" s="5" t="s">
+    <row r="10" spans="1:9" ht="90">
+      <c r="A10" s="4">
+        <v>5</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="103.2" customHeight="1">
+      <c r="A11" s="4">
+        <v>6</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="108">
+      <c r="A12" s="4">
+        <v>7</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="197.4" customHeight="1">
+      <c r="A13" s="4">
+        <v>8</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H8" s="11" t="s">
+      <c r="F13" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I13" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="90">
-      <c r="A9" s="4">
-        <v>5</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H9" s="11" t="s">
+    <row r="14" spans="1:9" ht="240.6" customHeight="1">
+      <c r="A14" s="16">
+        <v>9</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I14" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="103.2" customHeight="1">
-      <c r="A10" s="4">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="108">
-      <c r="A11" s="4">
-        <v>7</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="197.4" customHeight="1">
-      <c r="A12" s="4">
-        <v>8</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>6</v>
+    <row r="15" spans="1:9" ht="90">
+      <c r="A15" s="4">
+        <v>10</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="G15" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5" xr:uid="{E1472075-90BA-4648-91D3-5DF1C222D637}">
+  <autoFilter ref="A1:I5" xr:uid="{E1472075-90BA-4648-91D3-5DF1C222D637}">
     <filterColumn colId="1">
       <customFilters>
         <customFilter val="**"/>
@@ -3234,19 +3415,19 @@
     </filterColumn>
   </autoFilter>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:I4"/>
   </mergeCells>
-  <conditionalFormatting sqref="H3 H5:H12">
+  <conditionalFormatting sqref="I3 I5:I15">
     <cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="Failed">
-      <formula>NOT(ISERROR(SEARCH("Failed",H3)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Failed",I3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3 G5:G12" xr:uid="{7D86FEB8-93F1-4BDD-B501-493BB91A0C71}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3 H5:H15" xr:uid="{7D86FEB8-93F1-4BDD-B501-493BB91A0C71}">
       <formula1>"High, Medium, Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3 H5:H12" xr:uid="{18DB27D2-3E68-4DE7-97BA-86138D811D2E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3 I5:I15" xr:uid="{18DB27D2-3E68-4DE7-97BA-86138D811D2E}">
       <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3273,13 +3454,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
@@ -3297,22 +3478,22 @@
     <row r="2" spans="1:8" s="1" customFormat="1" ht="198">
       <c r="A2" s="19"/>
       <c r="B2" s="20" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H2" s="11" t="s">
         <v>12</v>
@@ -3323,19 +3504,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>7</v>
@@ -3349,16 +3530,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="10"/>
@@ -3369,22 +3550,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>6</v>
@@ -3395,22 +3576,22 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>6</v>
@@ -3421,22 +3602,22 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>6</v>
@@ -3447,22 +3628,22 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>6</v>
@@ -3473,22 +3654,22 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>6</v>
@@ -3533,13 +3714,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
@@ -3559,19 +3740,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -3585,22 +3766,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H3" s="11" t="s">
         <v>6</v>
@@ -4054,13 +4235,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
@@ -4080,16 +4261,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
@@ -4139,13 +4320,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
@@ -4165,16 +4346,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
@@ -4222,13 +4403,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>2</v>
@@ -4248,19 +4429,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -4307,13 +4488,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
@@ -4333,19 +4514,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -4392,13 +4573,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
@@ -4418,16 +4599,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="10" t="s">

</xml_diff>

<commit_message>
update file register test case
</commit_message>
<xml_diff>
--- a/manual_test/DuyenNTK Flashcard System Test Case.xlsx
+++ b/manual_test/DuyenNTK Flashcard System Test Case.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Learning24\web\learn-writing-english\manual_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57269D8-17FA-425E-9E72-A88C9044CB75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66CC14C5-B56E-4DC9-8407-F92D65ADC20E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Delete Note'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Download file'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log In'!$A$1:$I$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Register!$A$1:$I$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Register!$A$1:$I$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Remove all cards'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Remove all notes'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Search card'!$A$1:$H$2</definedName>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="190">
   <si>
     <t>N/A</t>
   </si>
@@ -79,11 +79,6 @@
   </si>
   <si>
     <t>High</t>
-  </si>
-  <si>
-    <t>1.Users access the system
-2.All fields are blank
-3.Click on &lt;ĐĂNG KÝ&gt; button</t>
   </si>
   <si>
     <t>1.Register screen is displayed
@@ -92,11 +87,6 @@
  - The system shows message: "Không được để trống"</t>
   </si>
   <si>
-    <t>1.Users access the system
-2.[username] field is blank
-3.Click on &lt;ĐĂNG KÝ&gt; button</t>
-  </si>
-  <si>
     <t>1.Register screen is displayed
 2.Data is inputted
 3.User sign up unsuccessfully
@@ -106,11 +96,6 @@
     <t>Failed</t>
   </si>
   <si>
-    <t>1.Users access the system
-2.[email] field is blank
-3.Click on &lt;ĐĂNG KÝ&gt; button</t>
-  </si>
-  <si>
     <t>Actual</t>
   </si>
   <si>
@@ -118,16 +103,6 @@
   </si>
   <si>
     <t>The system shows message: "Đăng ký thành công"</t>
-  </si>
-  <si>
-    <t>1.Users access the system
-2.[password] field is blank
-3.Click on &lt;ĐĂNG KÝ&gt; button</t>
-  </si>
-  <si>
-    <t>1.Users access the system
-2.[password] field length is less than 8
-3.Click on &lt;ĐĂNG KÝ&gt; button</t>
   </si>
   <si>
     <t>1.Register screen is displayed
@@ -140,11 +115,6 @@
   </si>
   <si>
     <t>The system shows message: "Không được để trống"</t>
-  </si>
-  <si>
-    <t>1.Users access the system
-2.[email] field is invalid
-3.Click on &lt;ĐĂNG KÝ&gt; button</t>
   </si>
   <si>
     <t>1.Register screen is displayed
@@ -846,6 +816,104 @@
     <t>1.Users access the system
 2.[email] field is valid, [password] field is wrong
 3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.All fields are blank
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[username] field is blank
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[email] field is blank
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[password] field is blank
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[password] field length is less than 8
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[email] field is invalid
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>[FlashCard][Register][Function]Register account unsuccessfully, in case:
+- Length [username] field &lt; 5</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.Length [username] field &lt; 5
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>1.Register screen is displayed
+2.Data is inputted
+3.User sign up unsuccessfully
+ - The system shows message: "Ít nhất 5 ký tự hoặc hơn!!!"</t>
+  </si>
+  <si>
+    <t>The system shows message: "Ít nhất 5 ký tự hoặc hơn!!!"</t>
+  </si>
+  <si>
+    <t>username: duyen0205
+email: testapp@gmail.com
+password: 12345678</t>
+  </si>
+  <si>
+    <t>username:
+ + a
+ + ab
+ + abc
+ + abcd</t>
+  </si>
+  <si>
+    <t>[FlashCard][Register][Function]Register account unsuccessfully, in case:
+- [username] field inputs special characters</t>
+  </si>
+  <si>
+    <t>username:
+ + @@@@@
+ + #####</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.[username] field inputs special characters
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>1.Register screen is displayed
+2.Data is inputted
+3.User sign up unsuccessfully
+ - The system shows message: "Username không chứa kí tự đặc biệt!!!"</t>
+  </si>
+  <si>
+    <t>Full email:
+ + abc_def-123@gmail-server.org
+ + user.name@example.co.uk
+ + rrrrrrrrrrrrrr@gmail.com
+ + 1111111111@gmail.com
+ + quoted.local@example.com
+ + contact@sub.domain.net
+ + user@.com
+ + user@com
+ + user@@example.com
+ + user..name@example.com
+ + user@example.com
+ + firstname.lastname@company.com
+ + admin@[192.168.1.1]
+ + user.@example.com
+ + user@192.168.1.999</t>
   </si>
 </sst>
 </file>
@@ -1078,6 +1146,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1089,9 +1160,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1652,15 +1720,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="57.33203125" style="1" customWidth="1"/>
-    <col min="3" max="4" width="43.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="43.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="51.44140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="47" style="1" customWidth="1"/>
     <col min="6" max="6" width="45.44140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="23.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="38.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="17.109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="17.77734375" style="1" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="1"/>
@@ -1671,22 +1740,22 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>3</v>
@@ -1700,20 +1769,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="5"/>
+        <v>52</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>183</v>
+      </c>
       <c r="E2" s="6" t="s">
         <v>5</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>7</v>
@@ -1727,23 +1798,23 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>9</v>
-      </c>
       <c r="G3" s="6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I3" s="11" t="s">
         <v>6</v>
@@ -1754,23 +1825,23 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="6" t="s">
-        <v>10</v>
+        <v>174</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I4" s="11" t="s">
         <v>6</v>
@@ -1781,122 +1852,182 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>69</v>
+        <v>179</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="5"/>
+        <v>52</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>184</v>
+      </c>
       <c r="E5" s="6" t="s">
-        <v>13</v>
+        <v>180</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>11</v>
+        <v>181</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>15</v>
+        <v>182</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="90">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="108">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>70</v>
+        <v>185</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="5"/>
+        <v>52</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>186</v>
+      </c>
       <c r="E6" s="6" t="s">
-        <v>17</v>
+        <v>187</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>11</v>
+        <v>188</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>21</v>
+        <v>161</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="108">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="90">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="6" t="s">
-        <v>18</v>
+        <v>175</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="108">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="90">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>159</v>
+        <v>64</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="6" t="s">
-        <v>22</v>
+        <v>176</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I8" s="11" t="s">
         <v>6</v>
       </c>
     </row>
+    <row r="9" spans="1:9" ht="108">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="299.39999999999998" customHeight="1">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I8" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}"/>
+  <autoFilter ref="A1:I10" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}"/>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="I2:I8">
+  <conditionalFormatting sqref="I2:I10">
     <cfRule type="containsText" dxfId="12" priority="7" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I8" xr:uid="{0FBBFA33-30F5-4E0C-9516-B35814C9A72D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I10" xr:uid="{0FBBFA33-30F5-4E0C-9516-B35814C9A72D}">
       <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H8" xr:uid="{455278D2-97C7-4EB1-A089-10A454F8270A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H10" xr:uid="{455278D2-97C7-4EB1-A089-10A454F8270A}">
       <formula1>"High, Medium, Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1923,19 +2054,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -1947,25 +2078,25 @@
     <row r="2" spans="1:8" s="1" customFormat="1" ht="283.2" customHeight="1">
       <c r="A2" s="19"/>
       <c r="B2" s="20" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="150" customHeight="1">
@@ -1973,19 +2104,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>7</v>
@@ -1999,22 +2130,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>6</v>
@@ -2025,22 +2156,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>6</v>
@@ -2051,22 +2182,22 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>6</v>
@@ -2341,19 +2472,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -2367,19 +2498,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2393,22 +2524,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H3" s="11" t="s">
         <v>6</v>
@@ -2691,19 +2822,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>3</v>
@@ -2717,19 +2848,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -2776,19 +2907,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -2802,16 +2933,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
@@ -2858,44 +2989,44 @@
   <sheetData>
     <row r="2" spans="6:12">
       <c r="F2" s="2"/>
-      <c r="G2" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
+      <c r="G2" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
     </row>
     <row r="3" spans="6:12">
       <c r="F3" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="4" spans="6:12">
       <c r="F4" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>0</v>
@@ -2915,13 +3046,13 @@
     </row>
     <row r="5" spans="6:12">
       <c r="F5" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>0</v>
@@ -2938,7 +3069,7 @@
     </row>
     <row r="6" spans="6:12">
       <c r="F6" s="3" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>0</v>
@@ -2947,13 +3078,13 @@
         <v>0</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>0</v>
@@ -2961,7 +3092,7 @@
     </row>
     <row r="7" spans="6:12">
       <c r="F7" s="3" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>0</v>
@@ -2973,7 +3104,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>0</v>
@@ -2984,7 +3115,7 @@
     </row>
     <row r="8" spans="6:12">
       <c r="F8" s="3" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>0</v>
@@ -3002,7 +3133,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -3036,22 +3167,22 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>3</v>
@@ -3061,68 +3192,68 @@
       </c>
     </row>
     <row r="2" spans="1:9" hidden="1">
-      <c r="A2" s="22"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="24"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="25"/>
     </row>
     <row r="3" spans="1:9" ht="162">
       <c r="A3" s="4"/>
       <c r="B3" s="5" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I3" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:9" hidden="1">
-      <c r="A4" s="22"/>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="24"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="25"/>
     </row>
     <row r="5" spans="1:9" ht="94.8" customHeight="1">
       <c r="A5" s="4">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G5" s="6"/>
       <c r="H5" s="10" t="s">
@@ -3137,23 +3268,23 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>171</v>
-      </c>
       <c r="F6" s="6" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I6" s="11" t="s">
         <v>6</v>
@@ -3161,23 +3292,23 @@
     </row>
     <row r="7" spans="1:9" ht="246.6" customHeight="1">
       <c r="A7" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="6" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>7</v>
@@ -3188,26 +3319,26 @@
     </row>
     <row r="8" spans="1:9" ht="90">
       <c r="A8" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="6" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I8" s="11" t="s">
         <v>6</v>
@@ -3215,26 +3346,26 @@
     </row>
     <row r="9" spans="1:9" ht="90">
       <c r="A9" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="6" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I9" s="11" t="s">
         <v>6</v>
@@ -3242,26 +3373,26 @@
     </row>
     <row r="10" spans="1:9" ht="90">
       <c r="A10" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="6" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I10" s="11" t="s">
         <v>6</v>
@@ -3269,26 +3400,26 @@
     </row>
     <row r="11" spans="1:9" ht="103.2" customHeight="1">
       <c r="A11" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="6" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I11" s="11" t="s">
         <v>6</v>
@@ -3296,26 +3427,26 @@
     </row>
     <row r="12" spans="1:9" ht="108">
       <c r="A12" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="6" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>6</v>
@@ -3323,23 +3454,23 @@
     </row>
     <row r="13" spans="1:9" ht="197.4" customHeight="1">
       <c r="A13" s="4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="6" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>7</v>
@@ -3350,28 +3481,28 @@
     </row>
     <row r="14" spans="1:9" ht="240.6" customHeight="1">
       <c r="A14" s="16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>168</v>
-      </c>
       <c r="E14" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="I14" s="11" t="s">
         <v>6</v>
@@ -3379,31 +3510,31 @@
     </row>
     <row r="15" spans="1:9" ht="90">
       <c r="A15" s="4">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I15" s="11" t="s">
         <v>10</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="G15" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -3454,19 +3585,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -3478,25 +3609,25 @@
     <row r="2" spans="1:8" s="1" customFormat="1" ht="198">
       <c r="A2" s="19"/>
       <c r="B2" s="20" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="199.8" customHeight="1">
@@ -3504,19 +3635,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>7</v>
@@ -3530,16 +3661,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="10"/>
@@ -3550,22 +3681,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>6</v>
@@ -3576,22 +3707,22 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>6</v>
@@ -3602,22 +3733,22 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="E7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>48</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>6</v>
@@ -3628,22 +3759,22 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>6</v>
@@ -3654,22 +3785,22 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>6</v>
@@ -3714,19 +3845,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -3740,19 +3871,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -3766,22 +3897,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H3" s="11" t="s">
         <v>6</v>
@@ -4235,19 +4366,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -4261,16 +4392,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
@@ -4320,19 +4451,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -4346,16 +4477,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
@@ -4403,19 +4534,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>3</v>
@@ -4429,19 +4560,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -4488,19 +4619,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -4514,19 +4645,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>7</v>
@@ -4573,19 +4704,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -4599,16 +4730,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="10" t="s">

</xml_diff>

<commit_message>
update file log in and sign up pages
</commit_message>
<xml_diff>
--- a/manual_test/DuyenNTK Flashcard System Test Case.xlsx
+++ b/manual_test/DuyenNTK Flashcard System Test Case.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Learning24\web\learn-writing-english\manual_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00662B18-8264-447A-897B-352900248193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A98B521-5453-48D5-8E2E-0AF6F3DB128C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F6133DD5-AC9E-4099-832C-9D6FC3656B2A}"/>
   </bookViews>
@@ -35,7 +35,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Delete Note'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Download file'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log In'!$A$1:$I$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Register!$A$1:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Register!$A$1:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Remove all cards'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Remove all notes'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Search card'!$A$1:$H$2</definedName>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="195">
   <si>
     <t>N/A</t>
   </si>
@@ -68,11 +68,6 @@
   </si>
   <si>
     <t>Status</t>
-  </si>
-  <si>
-    <t>1.Users access the system
-2.Input valid data into all fields
-3.Click on &lt;ĐĂNG KÝ&gt; button</t>
   </si>
   <si>
     <t>Passed</t>
@@ -121,11 +116,6 @@
 2.Data is inputted
 3.User sign up unsuccessfully
  - The system shows message: "Định dạng email không hợp lệ!"</t>
-  </si>
-  <si>
-    <t>1.Users access the system
-2.Input valid data into all fields
-3.Click on &lt;ĐĂNG NHẬP&gt; button</t>
   </si>
   <si>
     <t>1.Log In screen is displayed
@@ -615,14 +605,6 @@
     <t>1.The list card shows all cards
 2.The system remove all cards in UI &amp; database.
  + The number of cards has decreased on the badge.</t>
-  </si>
-  <si>
-    <t>1.Register screen is displayed
-2.Data is inputted
-3.User sign up successfully
- - The system shows message: "Đăng ký thành công"
- - Receive access_token
- - Navigate to log in page</t>
   </si>
   <si>
     <t>[FlashCard][Create Note][Function]Create a unsuccessful note, in case:
@@ -770,19 +752,6 @@
  + user@exam_ple.com</t>
   </si>
   <si>
-    <t>[FlashCard][Log In][Function]Log in successfully
- - Click on &lt;ĐĂNG NHẬP&gt; button + success</t>
-  </si>
-  <si>
-    <t>[FlashCard][Log In][Function]Log in successfully
- - Press enter &lt;ĐĂNG NHẬP&gt; button + success</t>
-  </si>
-  <si>
-    <t>1.Users access the system
-2.Click [email] field inputs data --&gt; enter --&gt; [password] field inputs data
-3.Press enter &lt;ĐĂNG NHẬP&gt; button</t>
-  </si>
-  <si>
     <t>1.Users access the system
 2.[email] field is blank
 3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
@@ -876,12 +845,6 @@
     <t>1.Users access the system
 2.[username] field inputs special characters
 3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
-  </si>
-  <si>
-    <t>1.Register screen is displayed
-2.Data is inputted
-3.User sign up unsuccessfully
- - The system shows message: "Username không chứa kí tự đặc biệt!!!"</t>
   </si>
   <si>
     <t>Full email:
@@ -916,6 +879,67 @@
  + #####
  + abc@1
  + #test</t>
+  </si>
+  <si>
+    <t>[FlashCard][Register][Function]Register account unsuccessfully, in case:
+- Length [username] field &gt; 20</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.Length [username] field &gt; 20
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>username:
+ + UserName2026SampleXYZ9e
+ + 1111222233334444555567</t>
+  </si>
+  <si>
+    <t>1.Register screen is displayed
+2.Data is inputted
+3.User sign up unsuccessfully
+ - The system shows message: "Tối đa 20 ký tự!!!"</t>
+  </si>
+  <si>
+    <t>The system shows message: "Tối đa 20 ký tự!!!"</t>
+  </si>
+  <si>
+    <t>1.Register screen is displayed
+2.Data is inputted
+3.User sign up unsuccessfully
+ - The system shows message: "Username chỉ được chứa chữ, số hoặc kết hợp giữa chữ và số, không phân biệt chữ hoa và chữ thường."</t>
+  </si>
+  <si>
+    <t>The system shows message: "Username chỉ được chứa chữ, số hoặc kết hợp giữa chữ và số, không phân biệt chữ hoa và chữ thường."</t>
+  </si>
+  <si>
+    <t>1.Register screen is displayed
+ - [username] field is auto focus
+2.Data is inputted
+3.User sign up successfully
+ - The system shows message: "Đăng ký thành công"
+ - Receive access_token
+ - Navigate to log in page</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+2.Input valid data into all fields
+3.Click / press enter &lt;ĐĂNG KÝ&gt; button</t>
+  </si>
+  <si>
+    <t>1.Users access the system
+  - [email] field is auto focus
+2.Input valid data into all fields
+3.Click / press enter &lt;ĐĂNG NHẬP&gt; button</t>
+  </si>
+  <si>
+    <t>email: testapp@gmail.com
+password: 12345678</t>
+  </si>
+  <si>
+    <t>[FlashCard][Log In][Function]Log in successfully, in case:
+ - All fields are valid
+ - Navigate to form page</t>
   </si>
 </sst>
 </file>
@@ -1722,11 +1746,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="57.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="60.44140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="43.5546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="51.44140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="47" style="1" customWidth="1"/>
@@ -1742,22 +1766,22 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>3</v>
@@ -1766,33 +1790,33 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="126">
+    <row r="2" spans="1:9" ht="162">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="11" t="s">
         <v>5</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="90">
@@ -1800,26 +1824,26 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="90">
@@ -1827,26 +1851,26 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="6" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="90">
@@ -1854,31 +1878,31 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="E5" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>187</v>
-      </c>
       <c r="G5" s="6" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="108">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="90">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1886,52 +1910,54 @@
         <v>183</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>184</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>161</v>
+        <v>187</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="90">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="144">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>63</v>
+        <v>177</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D7" s="5"/>
+        <v>50</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>182</v>
+      </c>
       <c r="E7" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>9</v>
+        <v>188</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>12</v>
+        <v>189</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="90">
@@ -1939,97 +1965,124 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="6" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="F8" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="108">
+    </row>
+    <row r="9" spans="1:9" ht="90">
       <c r="A9" s="4">
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="6" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>15</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="299.39999999999998" customHeight="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="108">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>153</v>
+        <v>63</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>186</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="D10" s="5"/>
       <c r="E10" s="6" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="299.39999999999998" customHeight="1">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I10" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}"/>
+  <autoFilter ref="A1:I11" xr:uid="{5679F970-FDE3-40AA-B766-39BAC6FA0D6E}"/>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="I2:I10">
+  <conditionalFormatting sqref="I2:I11">
     <cfRule type="containsText" dxfId="12" priority="7" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I10" xr:uid="{0FBBFA33-30F5-4E0C-9516-B35814C9A72D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I11" xr:uid="{0FBBFA33-30F5-4E0C-9516-B35814C9A72D}">
       <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H10" xr:uid="{455278D2-97C7-4EB1-A089-10A454F8270A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H11" xr:uid="{455278D2-97C7-4EB1-A089-10A454F8270A}">
       <formula1>"High, Medium, Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2056,19 +2109,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -2080,25 +2133,25 @@
     <row r="2" spans="1:8" s="1" customFormat="1" ht="283.2" customHeight="1">
       <c r="A2" s="19"/>
       <c r="B2" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="C2" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>142</v>
-      </c>
       <c r="E2" s="21" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="150" customHeight="1">
@@ -2106,25 +2159,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>97</v>
-      </c>
       <c r="G3" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="126">
@@ -2132,25 +2185,25 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>105</v>
-      </c>
       <c r="G4" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="139.80000000000001" customHeight="1">
@@ -2158,25 +2211,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>109</v>
-      </c>
       <c r="G5" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="180">
@@ -2184,25 +2237,25 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>135</v>
-      </c>
       <c r="G6" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18">
@@ -2474,19 +2527,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -2500,25 +2553,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D2" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>113</v>
-      </c>
       <c r="G2" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="180">
@@ -2526,25 +2579,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>118</v>
-      </c>
       <c r="G3" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18">
@@ -2824,19 +2877,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="14" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="14" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>3</v>
@@ -2850,25 +2903,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>146</v>
-      </c>
       <c r="G2" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2909,19 +2962,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -2935,23 +2988,23 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D2" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>121</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2992,7 +3045,7 @@
     <row r="2" spans="6:12">
       <c r="F2" s="2"/>
       <c r="G2" s="26" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H2" s="26"/>
       <c r="I2" s="26"/>
@@ -3002,33 +3055,33 @@
     </row>
     <row r="3" spans="6:12">
       <c r="F3" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="4" spans="6:12">
       <c r="F4" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>0</v>
@@ -3048,13 +3101,13 @@
     </row>
     <row r="5" spans="6:12">
       <c r="F5" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>0</v>
@@ -3071,7 +3124,7 @@
     </row>
     <row r="6" spans="6:12">
       <c r="F6" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>0</v>
@@ -3080,13 +3133,13 @@
         <v>0</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>0</v>
@@ -3094,7 +3147,7 @@
     </row>
     <row r="7" spans="6:12">
       <c r="F7" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>0</v>
@@ -3106,7 +3159,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>0</v>
@@ -3117,7 +3170,7 @@
     </row>
     <row r="8" spans="6:12">
       <c r="F8" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>0</v>
@@ -3135,7 +3188,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -3150,13 +3203,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1472075-90BA-4648-91D3-5DF1C222D637}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
     <col min="2" max="2" width="53" style="1" customWidth="1"/>
     <col min="3" max="4" width="42.5546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="47.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="54.5546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="58.44140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="50.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="16.5546875" style="1" customWidth="1"/>
@@ -3169,22 +3222,22 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>3</v>
@@ -3207,24 +3260,24 @@
     <row r="3" spans="1:9" ht="162">
       <c r="A3" s="4"/>
       <c r="B3" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:9" hidden="1">
@@ -3238,305 +3291,278 @@
       <c r="H4" s="24"/>
       <c r="I4" s="25"/>
     </row>
-    <row r="5" spans="1:9" ht="94.8" customHeight="1">
+    <row r="5" spans="1:9" ht="113.4" customHeight="1">
       <c r="A5" s="4">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>163</v>
+        <v>194</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>159</v>
+        <v>193</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>18</v>
+        <v>192</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G5" s="6"/>
       <c r="H5" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I5" s="11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="246.6" customHeight="1">
+      <c r="A6" s="4">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H6" s="10" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" ht="109.2" customHeight="1">
-      <c r="A6" s="4">
-        <v>2</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G6" s="6"/>
-      <c r="H6" s="10" t="s">
-        <v>48</v>
-      </c>
       <c r="I6" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="246.6" customHeight="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="90">
       <c r="A7" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="6" t="s">
-        <v>59</v>
+        <v>161</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>81</v>
+        <v>17</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="90">
       <c r="A8" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="6" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="90">
       <c r="A9" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="6" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="90">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="103.2" customHeight="1">
       <c r="A10" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="6" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="103.2" customHeight="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="108">
       <c r="A11" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="6" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>15</v>
+        <v>76</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="108">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="197.4" customHeight="1">
       <c r="A12" s="4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>57</v>
+        <v>108</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="6" t="s">
-        <v>170</v>
+        <v>57</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" s="6" t="s">
         <v>78</v>
       </c>
+      <c r="G12" s="5" t="s">
+        <v>77</v>
+      </c>
       <c r="H12" s="10" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="197.4" customHeight="1">
-      <c r="A13" s="4">
-        <v>9</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="240.6" customHeight="1">
+      <c r="A13" s="16">
+        <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>110</v>
+        <v>152</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="D13" s="5"/>
+        <v>153</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>159</v>
+      </c>
       <c r="E13" s="6" t="s">
-        <v>59</v>
+        <v>165</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>80</v>
+        <v>154</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>79</v>
+        <v>11</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="240.6" customHeight="1">
-      <c r="A14" s="16">
-        <v>10</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="90">
+      <c r="A14" s="4">
+        <v>11</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>155</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="E14" s="6" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>12</v>
+      <c r="G14" s="22" t="s">
+        <v>158</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="90">
-      <c r="A15" s="4">
-        <v>11</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="G15" s="22" t="s">
-        <v>161</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -3551,16 +3577,16 @@
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:I4"/>
   </mergeCells>
-  <conditionalFormatting sqref="I3 I5:I15">
+  <conditionalFormatting sqref="I3 I5:I14">
     <cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",I3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3 H5:H15" xr:uid="{7D86FEB8-93F1-4BDD-B501-493BB91A0C71}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3 H5:H14" xr:uid="{7D86FEB8-93F1-4BDD-B501-493BB91A0C71}">
       <formula1>"High, Medium, Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3 I5:I15" xr:uid="{18DB27D2-3E68-4DE7-97BA-86138D811D2E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3 I5:I14" xr:uid="{18DB27D2-3E68-4DE7-97BA-86138D811D2E}">
       <formula1>"Passed,Failed,Untested,Accepted,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3587,19 +3613,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -3611,25 +3637,25 @@
     <row r="2" spans="1:8" s="1" customFormat="1" ht="198">
       <c r="A2" s="19"/>
       <c r="B2" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="F2" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="C2" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="E2" s="20" t="s">
-        <v>150</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>151</v>
-      </c>
       <c r="G2" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="199.8" customHeight="1">
@@ -3637,25 +3663,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="90">
@@ -3663,16 +3689,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>99</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>101</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="10"/>
@@ -3683,25 +3709,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="90">
@@ -3709,25 +3735,25 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="108">
@@ -3735,25 +3761,25 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="108">
@@ -3761,25 +3787,25 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="108">
@@ -3787,25 +3813,25 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3847,19 +3873,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -3873,25 +3899,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="90">
@@ -3899,25 +3925,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>48</v>
-      </c>
       <c r="H3" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18">
@@ -4368,19 +4394,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -4394,23 +4420,23 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -4453,19 +4479,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -4479,23 +4505,23 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>125</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>127</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -4536,19 +4562,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="14" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="14" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>3</v>
@@ -4562,25 +4588,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -4621,19 +4647,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -4647,25 +4673,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>91</v>
-      </c>
       <c r="G2" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -4706,19 +4732,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>51</v>
-      </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>3</v>
@@ -4732,23 +4758,23 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>